<commit_message>
Updated ReadMe to specify asset files in Releases; updated P/N for chassis in BOM
</commit_message>
<xml_diff>
--- a/dVRK-Si-Controller-BOM.xlsx
+++ b/dVRK-Si-Controller-BOM.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Peter\JHU\Hardware\ControllerBuild\dVRK-S\mfg-process\dVRK-Si-Controller\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98BDEA04-7DEF-4573-A3C4-95ED358DF8C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9192"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Controller" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -201,9 +207,6 @@
     <t>Top panel screws provided by Protocase</t>
   </si>
   <si>
-    <t>165597-1</t>
-  </si>
-  <si>
     <t>Design Files</t>
   </si>
   <si>
@@ -421,12 +424,15 @@
   </si>
   <si>
     <t>Lower cost alternative is Amphenol TS06315A0000G (Digikey P/N 609-3790-ND)</t>
+  </si>
+  <si>
+    <t>dVRK Si Controller Chassis Rev 3</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -907,7 +913,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
@@ -920,14 +926,14 @@
     <col min="3" max="3" width="44.33203125" customWidth="1"/>
     <col min="4" max="4" width="9.77734375" style="2" customWidth="1"/>
     <col min="5" max="5" width="17.21875" customWidth="1"/>
-    <col min="6" max="6" width="23.77734375" customWidth="1"/>
+    <col min="6" max="6" width="28.77734375" customWidth="1"/>
     <col min="7" max="7" width="15.77734375" customWidth="1"/>
     <col min="8" max="8" width="31.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="36.6" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B1" s="38" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C1" s="38"/>
       <c r="D1" s="38"/>
@@ -949,7 +955,7 @@
     </row>
     <row r="3" spans="1:8" ht="21" x14ac:dyDescent="0.4">
       <c r="B3" s="36">
-        <v>45889</v>
+        <v>45902</v>
       </c>
       <c r="C3" s="36"/>
       <c r="D3" s="36"/>
@@ -1026,7 +1032,7 @@
         <v>31</v>
       </c>
       <c r="F8" s="22" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G8" s="12" t="s">
         <v>17</v>
@@ -1041,14 +1047,14 @@
         <v>1</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D9" s="19"/>
       <c r="E9" s="12" t="s">
         <v>31</v>
       </c>
       <c r="F9" s="22" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G9" s="12" t="s">
         <v>17</v>
@@ -1063,17 +1069,17 @@
         <v>1</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D10" s="19"/>
       <c r="E10" s="12" t="s">
         <v>31</v>
       </c>
       <c r="F10" s="22" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H10" s="4"/>
     </row>
@@ -1159,7 +1165,7 @@
         <v>6</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D14" s="15"/>
       <c r="E14" s="12" t="s">
@@ -1229,18 +1235,18 @@
         <v>1</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D17" s="15"/>
       <c r="E17" s="12" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F17" s="6"/>
       <c r="G17" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="H17" s="31" t="s">
         <v>122</v>
-      </c>
-      <c r="H17" s="31" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1257,7 +1263,7 @@
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="23" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D19" s="19">
         <v>2</v>
@@ -1393,7 +1399,7 @@
       <c r="A28" s="14"/>
       <c r="B28" s="14"/>
       <c r="C28" s="27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D28" s="14"/>
       <c r="E28" s="4"/>
@@ -1407,7 +1413,7 @@
         <v>7</v>
       </c>
       <c r="C29" s="26" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D29" s="14"/>
       <c r="E29" s="26" t="s">
@@ -1418,7 +1424,7 @@
         <v>36</v>
       </c>
       <c r="H29" s="26" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1427,20 +1433,20 @@
         <v>3</v>
       </c>
       <c r="C30" s="26" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D30" s="14"/>
       <c r="E30" s="26" t="s">
         <v>43</v>
       </c>
       <c r="F30" s="26" t="s">
+        <v>65</v>
+      </c>
+      <c r="G30" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="H30" s="26" t="s">
         <v>66</v>
-      </c>
-      <c r="G30" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="H30" s="26" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1449,7 +1455,7 @@
         <v>4</v>
       </c>
       <c r="C31" s="26" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D31" s="14"/>
       <c r="E31" s="26" t="s">
@@ -1460,7 +1466,7 @@
         <v>36</v>
       </c>
       <c r="H31" s="26" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1469,20 +1475,20 @@
         <v>1</v>
       </c>
       <c r="C32" s="26" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D32" s="14"/>
       <c r="E32" s="26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F32" s="26" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G32" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H32" s="26" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1491,20 +1497,20 @@
         <v>2</v>
       </c>
       <c r="C33" s="26" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D33" s="14"/>
       <c r="E33" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="F33" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="F33" s="26" t="s">
+      <c r="G33" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="H33" s="26" t="s">
         <v>72</v>
-      </c>
-      <c r="G33" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="H33" s="26" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1513,20 +1519,20 @@
         <v>2</v>
       </c>
       <c r="C34" s="26" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D34" s="14"/>
       <c r="E34" s="26" t="s">
         <v>43</v>
       </c>
       <c r="F34" s="26" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G34" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H34" s="26" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1535,20 +1541,20 @@
         <v>2</v>
       </c>
       <c r="C35" s="26" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D35" s="14"/>
       <c r="E35" s="26" t="s">
         <v>43</v>
       </c>
       <c r="F35" s="26" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G35" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H35" s="26" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1557,20 +1563,20 @@
         <v>4</v>
       </c>
       <c r="C36" s="26" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D36" s="14"/>
       <c r="E36" s="26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F36" s="26" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G36" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H36" s="26" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1579,20 +1585,20 @@
         <v>1</v>
       </c>
       <c r="C37" s="26" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D37" s="14"/>
       <c r="E37" s="26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F37" s="26" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G37" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H37" s="26" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1601,20 +1607,20 @@
         <v>1</v>
       </c>
       <c r="C38" s="26" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D38" s="14"/>
       <c r="E38" s="26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F38" s="26" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G38" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H38" s="26" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1623,22 +1629,22 @@
         <v>1</v>
       </c>
       <c r="C39" s="26" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D39" s="14">
         <v>3</v>
       </c>
       <c r="E39" s="26" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F39" s="28" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G39" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H39" s="26" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1647,20 +1653,20 @@
         <v>2</v>
       </c>
       <c r="C40" s="26" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D40" s="14"/>
       <c r="E40" s="26" t="s">
+        <v>98</v>
+      </c>
+      <c r="F40" s="28" t="s">
         <v>99</v>
       </c>
-      <c r="F40" s="28" t="s">
-        <v>100</v>
-      </c>
       <c r="G40" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H40" s="26" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1669,20 +1675,20 @@
         <v>4</v>
       </c>
       <c r="C41" s="26" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D41" s="14"/>
       <c r="E41" s="26" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F41" s="26" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G41" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H41" s="26" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1691,20 +1697,20 @@
         <v>2</v>
       </c>
       <c r="C42" s="26" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D42" s="14"/>
       <c r="E42" s="26" t="s">
         <v>43</v>
       </c>
       <c r="F42" s="26" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G42" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H42" s="26" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1713,20 +1719,20 @@
         <v>2</v>
       </c>
       <c r="C43" s="26" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D43" s="14"/>
       <c r="E43" s="26" t="s">
         <v>43</v>
       </c>
       <c r="F43" s="26" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G43" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H43" s="26" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1746,7 +1752,7 @@
         <v>0</v>
       </c>
       <c r="D45" s="19" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E45" s="5"/>
       <c r="F45" s="4"/>
@@ -1761,7 +1767,7 @@
         <v>34</v>
       </c>
       <c r="C46" s="12" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D46" s="15"/>
       <c r="E46" s="12" t="s">
@@ -1779,7 +1785,7 @@
         <v>2</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D47" s="15"/>
       <c r="E47" s="12" t="s">
@@ -1797,7 +1803,7 @@
         <v>1</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D48" s="15"/>
       <c r="E48" s="12" t="s">
@@ -1815,7 +1821,7 @@
         <v>3</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D49" s="15"/>
       <c r="E49" s="12" t="s">
@@ -1877,14 +1883,14 @@
         <v>2</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D52" s="15"/>
       <c r="E52" s="12" t="s">
         <v>43</v>
       </c>
       <c r="F52" s="26" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G52" s="12" t="s">
         <v>36</v>
@@ -1901,14 +1907,14 @@
         <v>4</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D53" s="15"/>
       <c r="E53" s="12" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F53" s="26" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G53" s="12" t="s">
         <v>36</v>
@@ -1953,14 +1959,14 @@
       <c r="E56" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="F56" s="4" t="s">
-        <v>60</v>
+      <c r="F56" s="26" t="s">
+        <v>133</v>
       </c>
       <c r="G56" s="6" t="s">
         <v>20</v>
       </c>
       <c r="H56" s="26" t="s">
-        <v>60</v>
+        <v>133</v>
       </c>
     </row>
     <row r="57" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
@@ -1978,10 +1984,10 @@
         <v>31</v>
       </c>
       <c r="F57" s="26" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G57" s="12" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H57" s="4"/>
     </row>
@@ -1996,7 +2002,7 @@
         <v>1</v>
       </c>
       <c r="C60" s="25" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="61" spans="1:8" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2005,7 +2011,7 @@
         <v>2</v>
       </c>
       <c r="C61" s="25" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="62" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2013,7 +2019,7 @@
         <v>3</v>
       </c>
       <c r="C62" s="29" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="63" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
@@ -2047,9 +2053,9 @@
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="F10" r:id="rId1"/>
-    <hyperlink ref="F9" r:id="rId2"/>
-    <hyperlink ref="F8" r:id="rId3"/>
+    <hyperlink ref="F10" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="F9" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="F8" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="72" fitToHeight="0" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId4"/>

</xml_diff>

<commit_message>
Updates for Rev 4
</commit_message>
<xml_diff>
--- a/dVRK-Si-Controller-BOM.xlsx
+++ b/dVRK-Si-Controller-BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Peter\JHU\Hardware\ControllerBuild\dVRK-S\mfg-process\dVRK-Si-Controller\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98BDEA04-7DEF-4573-A3C4-95ED358DF8C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{485E9288-3F44-448B-9D10-67AF7971D8B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="143">
   <si>
     <t>Fasteners</t>
   </si>
@@ -417,16 +417,43 @@
     <t>See assembly instructions for wire/cable specifications</t>
   </si>
   <si>
-    <t>dVRK-Si Controller, Rev 1.0.1</t>
-  </si>
-  <si>
     <t>FPGA V3.x (x = 1 or 2)</t>
   </si>
   <si>
     <t>Lower cost alternative is Amphenol TS06315A0000G (Digikey P/N 609-3790-ND)</t>
   </si>
   <si>
-    <t>dVRK Si Controller Chassis Rev 3</t>
+    <t>dVRK-Si Controller, Rev 1.1.0</t>
+  </si>
+  <si>
+    <t>dVRK Aux I/O V1</t>
+  </si>
+  <si>
+    <t>JLCPCB</t>
+  </si>
+  <si>
+    <t>Wire harness assy, Aux I/O</t>
+  </si>
+  <si>
+    <t>Hirose</t>
+  </si>
+  <si>
+    <t>DF11-6DS-2C</t>
+  </si>
+  <si>
+    <t>H2021-ND</t>
+  </si>
+  <si>
+    <t>dVRK Si Controller Chassis Rev 4</t>
+  </si>
+  <si>
+    <t>H3BBT-10108-#8</t>
+  </si>
+  <si>
+    <t>Replace # by wire color (B=black, W=white, G=green, R=red, L=blue, A=amber)</t>
+  </si>
+  <si>
+    <t>Wire, Precrimped, 28 AWG, 8", multiple colors</t>
   </si>
 </sst>
 </file>
@@ -918,7 +945,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.44140625" style="2" customWidth="1"/>
@@ -933,7 +960,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="36.6" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B1" s="38" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C1" s="38"/>
       <c r="D1" s="38"/>
@@ -955,7 +982,7 @@
     </row>
     <row r="3" spans="1:8" ht="21" x14ac:dyDescent="0.4">
       <c r="B3" s="36">
-        <v>45902</v>
+        <v>46115</v>
       </c>
       <c r="C3" s="36"/>
       <c r="D3" s="36"/>
@@ -1047,7 +1074,7 @@
         <v>1</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D9" s="19"/>
       <c r="E9" s="12" t="s">
@@ -1249,55 +1276,61 @@
         <v>122</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="14"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
-    </row>
-    <row r="19" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A18" s="15">
+        <v>111</v>
+      </c>
+      <c r="B18" s="15">
+        <v>1</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="D18" s="15"/>
+      <c r="E18" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="F18" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="G18" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="H18" s="31"/>
+    </row>
+    <row r="19" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
-      <c r="C19" s="23" t="s">
-        <v>128</v>
-      </c>
-      <c r="D19" s="19">
-        <v>2</v>
-      </c>
-      <c r="E19" s="5"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="4"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
     </row>
     <row r="20" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A20" s="15">
-        <v>201</v>
-      </c>
-      <c r="B20" s="15">
+      <c r="A20" s="14"/>
+      <c r="B20" s="14"/>
+      <c r="C20" s="23" t="s">
+        <v>128</v>
+      </c>
+      <c r="D20" s="19">
         <v>2</v>
       </c>
-      <c r="C20" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="D20" s="15"/>
-      <c r="E20" s="6"/>
+      <c r="E20" s="5"/>
       <c r="F20" s="4"/>
-      <c r="G20" s="6"/>
+      <c r="G20" s="4"/>
       <c r="H20" s="4"/>
     </row>
     <row r="21" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A21" s="15">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B21" s="15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D21" s="15"/>
       <c r="E21" s="6"/>
@@ -1307,13 +1340,13 @@
     </row>
     <row r="22" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A22" s="15">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B22" s="15">
         <v>1</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D22" s="15"/>
       <c r="E22" s="6"/>
@@ -1323,13 +1356,13 @@
     </row>
     <row r="23" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A23" s="15">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B23" s="15">
         <v>1</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D23" s="15"/>
       <c r="E23" s="6"/>
@@ -1339,13 +1372,13 @@
     </row>
     <row r="24" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A24" s="15">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B24" s="15">
         <v>1</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D24" s="15"/>
       <c r="E24" s="6"/>
@@ -1355,13 +1388,13 @@
     </row>
     <row r="25" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A25" s="15">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B25" s="15">
         <v>1</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D25" s="15"/>
       <c r="E25" s="6"/>
@@ -1371,13 +1404,13 @@
     </row>
     <row r="26" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A26" s="15">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B26" s="15">
         <v>1</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D26" s="15"/>
       <c r="E26" s="6"/>
@@ -1385,154 +1418,142 @@
       <c r="G26" s="6"/>
       <c r="H26" s="4"/>
     </row>
-    <row r="27" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="14"/>
-      <c r="B27" s="14"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="4"/>
+    <row r="27" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A27" s="15">
+        <v>207</v>
+      </c>
+      <c r="B27" s="15">
+        <v>1</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="D27" s="15"/>
+      <c r="E27" s="6"/>
       <c r="F27" s="4"/>
-      <c r="G27" s="4"/>
+      <c r="G27" s="6"/>
       <c r="H27" s="4"/>
     </row>
-    <row r="28" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="14"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="27" t="s">
-        <v>119</v>
-      </c>
-      <c r="D28" s="14"/>
-      <c r="E28" s="4"/>
+    <row r="28" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A28" s="15">
+        <v>208</v>
+      </c>
+      <c r="B28" s="15">
+        <v>1</v>
+      </c>
+      <c r="C28" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="D28" s="15"/>
+      <c r="E28" s="6"/>
       <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
+      <c r="G28" s="6"/>
       <c r="H28" s="4"/>
     </row>
     <row r="29" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="14"/>
-      <c r="B29" s="14">
-        <v>7</v>
-      </c>
-      <c r="C29" s="26" t="s">
-        <v>67</v>
-      </c>
+      <c r="B29" s="14"/>
+      <c r="C29" s="4"/>
       <c r="D29" s="14"/>
-      <c r="E29" s="26" t="s">
-        <v>47</v>
-      </c>
+      <c r="E29" s="4"/>
       <c r="F29" s="4"/>
-      <c r="G29" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="H29" s="26" t="s">
-        <v>63</v>
-      </c>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4"/>
     </row>
     <row r="30" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="14"/>
-      <c r="B30" s="14">
-        <v>3</v>
-      </c>
-      <c r="C30" s="26" t="s">
-        <v>64</v>
+      <c r="B30" s="14"/>
+      <c r="C30" s="27" t="s">
+        <v>119</v>
       </c>
       <c r="D30" s="14"/>
-      <c r="E30" s="26" t="s">
-        <v>43</v>
-      </c>
-      <c r="F30" s="26" t="s">
-        <v>65</v>
-      </c>
-      <c r="G30" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="H30" s="26" t="s">
-        <v>66</v>
-      </c>
+      <c r="E30" s="4"/>
+      <c r="F30" s="4"/>
+      <c r="G30" s="4"/>
+      <c r="H30" s="4"/>
     </row>
     <row r="31" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="14"/>
       <c r="B31" s="14">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C31" s="26" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D31" s="14"/>
       <c r="E31" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="F31" s="26"/>
+      <c r="F31" s="4"/>
       <c r="G31" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H31" s="26" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="14"/>
       <c r="B32" s="14">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C32" s="26" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="D32" s="14"/>
       <c r="E32" s="26" t="s">
-        <v>70</v>
+        <v>43</v>
       </c>
       <c r="F32" s="26" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="G32" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H32" s="26" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="14"/>
       <c r="B33" s="14">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C33" s="26" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="D33" s="14"/>
       <c r="E33" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="F33" s="26" t="s">
-        <v>71</v>
-      </c>
+        <v>47</v>
+      </c>
+      <c r="F33" s="26"/>
       <c r="G33" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H33" s="26" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="14"/>
       <c r="B34" s="14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C34" s="26" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D34" s="14"/>
       <c r="E34" s="26" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="F34" s="26" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="G34" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H34" s="26" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1541,86 +1562,86 @@
         <v>2</v>
       </c>
       <c r="C35" s="26" t="s">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="D35" s="14"/>
       <c r="E35" s="26" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="F35" s="26" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="G35" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H35" s="26" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="14"/>
       <c r="B36" s="14">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C36" s="26" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="D36" s="14"/>
       <c r="E36" s="26" t="s">
-        <v>70</v>
+        <v>43</v>
       </c>
       <c r="F36" s="26" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="G36" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H36" s="26" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="14"/>
       <c r="B37" s="14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C37" s="26" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="D37" s="14"/>
       <c r="E37" s="26" t="s">
-        <v>70</v>
+        <v>43</v>
       </c>
       <c r="F37" s="26" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="G37" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H37" s="26" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="14"/>
       <c r="B38" s="14">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C38" s="26" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D38" s="14"/>
       <c r="E38" s="26" t="s">
         <v>70</v>
       </c>
       <c r="F38" s="26" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="G38" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H38" s="26" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1629,66 +1650,66 @@
         <v>1</v>
       </c>
       <c r="C39" s="26" t="s">
-        <v>94</v>
-      </c>
-      <c r="D39" s="14">
-        <v>3</v>
-      </c>
+        <v>86</v>
+      </c>
+      <c r="D39" s="14"/>
       <c r="E39" s="26" t="s">
-        <v>93</v>
-      </c>
-      <c r="F39" s="28" t="s">
-        <v>95</v>
+        <v>70</v>
+      </c>
+      <c r="F39" s="26" t="s">
+        <v>85</v>
       </c>
       <c r="G39" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H39" s="26" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="14"/>
       <c r="B40" s="14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C40" s="26" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="D40" s="14"/>
       <c r="E40" s="26" t="s">
-        <v>98</v>
-      </c>
-      <c r="F40" s="28" t="s">
-        <v>99</v>
+        <v>70</v>
+      </c>
+      <c r="F40" s="26" t="s">
+        <v>89</v>
       </c>
       <c r="G40" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H40" s="26" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="14"/>
       <c r="B41" s="14">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C41" s="26" t="s">
-        <v>101</v>
-      </c>
-      <c r="D41" s="14"/>
+        <v>94</v>
+      </c>
+      <c r="D41" s="14">
+        <v>3</v>
+      </c>
       <c r="E41" s="26" t="s">
-        <v>103</v>
-      </c>
-      <c r="F41" s="26" t="s">
-        <v>102</v>
+        <v>93</v>
+      </c>
+      <c r="F41" s="28" t="s">
+        <v>95</v>
       </c>
       <c r="G41" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H41" s="26" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1697,353 +1718,451 @@
         <v>2</v>
       </c>
       <c r="C42" s="26" t="s">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="D42" s="14"/>
       <c r="E42" s="26" t="s">
-        <v>43</v>
-      </c>
-      <c r="F42" s="26" t="s">
-        <v>105</v>
+        <v>98</v>
+      </c>
+      <c r="F42" s="28" t="s">
+        <v>99</v>
       </c>
       <c r="G42" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H42" s="26" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="14"/>
       <c r="B43" s="14">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C43" s="26" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="D43" s="14"/>
       <c r="E43" s="26" t="s">
-        <v>43</v>
+        <v>103</v>
       </c>
       <c r="F43" s="26" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="G43" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H43" s="26" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="14"/>
-      <c r="B44" s="14"/>
-      <c r="C44" s="26"/>
+      <c r="B44" s="14">
+        <v>2</v>
+      </c>
+      <c r="C44" s="26" t="s">
+        <v>106</v>
+      </c>
       <c r="D44" s="14"/>
-      <c r="E44" s="26"/>
-      <c r="F44" s="26"/>
-      <c r="G44" s="26"/>
-      <c r="H44" s="26"/>
-    </row>
-    <row r="45" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A45" s="16"/>
-      <c r="B45" s="14"/>
-      <c r="C45" s="5" t="s">
+      <c r="E44" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="F44" s="26" t="s">
+        <v>105</v>
+      </c>
+      <c r="G44" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="H44" s="26" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="14"/>
+      <c r="B45" s="14">
+        <v>2</v>
+      </c>
+      <c r="C45" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="D45" s="14"/>
+      <c r="E45" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="F45" s="26" t="s">
+        <v>107</v>
+      </c>
+      <c r="G45" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="H45" s="26" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="14"/>
+      <c r="B46" s="14">
+        <v>2</v>
+      </c>
+      <c r="C46" s="26" t="s">
+        <v>86</v>
+      </c>
+      <c r="D46" s="14"/>
+      <c r="E46" s="26" t="s">
+        <v>136</v>
+      </c>
+      <c r="F46" s="26" t="s">
+        <v>137</v>
+      </c>
+      <c r="G46" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="H46" s="26" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="14"/>
+      <c r="B47" s="14">
+        <v>6</v>
+      </c>
+      <c r="C47" s="26" t="s">
+        <v>142</v>
+      </c>
+      <c r="D47" s="14">
+        <v>7</v>
+      </c>
+      <c r="E47" s="26" t="s">
+        <v>136</v>
+      </c>
+      <c r="F47" s="26" t="s">
+        <v>140</v>
+      </c>
+      <c r="G47" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="H47" s="26" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="14"/>
+      <c r="B48" s="14"/>
+      <c r="C48" s="26"/>
+      <c r="D48" s="14"/>
+      <c r="E48" s="26"/>
+      <c r="F48" s="26"/>
+      <c r="G48" s="26"/>
+      <c r="H48" s="26"/>
+    </row>
+    <row r="49" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A49" s="16"/>
+      <c r="B49" s="14"/>
+      <c r="C49" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="D45" s="19" t="s">
+      <c r="D49" s="19" t="s">
         <v>124</v>
       </c>
-      <c r="E45" s="5"/>
-      <c r="F45" s="4"/>
-      <c r="G45" s="4"/>
-      <c r="H45" s="4"/>
-    </row>
-    <row r="46" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A46" s="15">
-        <v>301</v>
-      </c>
-      <c r="B46" s="15">
-        <v>34</v>
-      </c>
-      <c r="C46" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="D46" s="15"/>
-      <c r="E46" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="F46" s="4"/>
-      <c r="G46" s="4"/>
-      <c r="H46" s="4"/>
-    </row>
-    <row r="47" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A47" s="15">
-        <v>302</v>
-      </c>
-      <c r="B47" s="15">
-        <v>2</v>
-      </c>
-      <c r="C47" s="12" t="s">
-        <v>115</v>
-      </c>
-      <c r="D47" s="15"/>
-      <c r="E47" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="F47" s="4"/>
-      <c r="G47" s="4"/>
-      <c r="H47" s="4"/>
-    </row>
-    <row r="48" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A48" s="15">
-        <v>303</v>
-      </c>
-      <c r="B48" s="15">
-        <v>1</v>
-      </c>
-      <c r="C48" s="12" t="s">
-        <v>116</v>
-      </c>
-      <c r="D48" s="15"/>
-      <c r="E48" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="F48" s="4"/>
-      <c r="G48" s="4"/>
-      <c r="H48" s="4"/>
-    </row>
-    <row r="49" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A49" s="15">
-        <v>304</v>
-      </c>
-      <c r="B49" s="15">
-        <v>3</v>
-      </c>
-      <c r="C49" s="12" t="s">
-        <v>117</v>
-      </c>
-      <c r="D49" s="15"/>
-      <c r="E49" s="12" t="s">
-        <v>47</v>
-      </c>
+      <c r="E49" s="5"/>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
       <c r="H49" s="4"/>
     </row>
     <row r="50" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A50" s="15">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="B50" s="15">
-        <v>3</v>
-      </c>
-      <c r="C50" s="6" t="s">
-        <v>1</v>
+        <v>34</v>
+      </c>
+      <c r="C50" s="12" t="s">
+        <v>114</v>
       </c>
       <c r="D50" s="15"/>
       <c r="E50" s="12" t="s">
         <v>47</v>
       </c>
       <c r="F50" s="4"/>
-      <c r="G50" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="H50" s="12" t="s">
-        <v>3</v>
-      </c>
+      <c r="G50" s="4"/>
+      <c r="H50" s="4"/>
     </row>
     <row r="51" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A51" s="15">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="B51" s="15">
-        <v>1</v>
-      </c>
-      <c r="C51" s="6" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C51" s="12" t="s">
+        <v>115</v>
       </c>
       <c r="D51" s="15"/>
       <c r="E51" s="12" t="s">
         <v>47</v>
       </c>
       <c r="F51" s="4"/>
-      <c r="G51" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="H51" s="12" t="s">
-        <v>5</v>
-      </c>
+      <c r="G51" s="4"/>
+      <c r="H51" s="4"/>
     </row>
     <row r="52" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A52" s="15">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="B52" s="15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="D52" s="15"/>
       <c r="E52" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="F52" s="26" t="s">
-        <v>109</v>
-      </c>
-      <c r="G52" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="H52" s="12" t="s">
-        <v>6</v>
-      </c>
+        <v>47</v>
+      </c>
+      <c r="F52" s="4"/>
+      <c r="G52" s="4"/>
+      <c r="H52" s="4"/>
     </row>
     <row r="53" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A53" s="15">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="B53" s="15">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="D53" s="15"/>
       <c r="E53" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="F53" s="26" t="s">
-        <v>112</v>
-      </c>
-      <c r="G53" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="H53" s="12" t="s">
-        <v>7</v>
-      </c>
+        <v>47</v>
+      </c>
+      <c r="F53" s="4"/>
+      <c r="G53" s="4"/>
+      <c r="H53" s="4"/>
     </row>
     <row r="54" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A54" s="14"/>
-      <c r="B54" s="14"/>
-      <c r="C54" s="7"/>
-      <c r="D54" s="20"/>
-      <c r="E54" s="7"/>
+      <c r="A54" s="15">
+        <v>305</v>
+      </c>
+      <c r="B54" s="15">
+        <v>3</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D54" s="15"/>
+      <c r="E54" s="12" t="s">
+        <v>47</v>
+      </c>
       <c r="F54" s="4"/>
-      <c r="G54" s="4"/>
-      <c r="H54" s="4"/>
+      <c r="G54" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="H54" s="12" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="55" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A55" s="14"/>
-      <c r="B55" s="14"/>
-      <c r="C55" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D55" s="16"/>
-      <c r="E55" s="5"/>
+      <c r="A55" s="15">
+        <v>306</v>
+      </c>
+      <c r="B55" s="15">
+        <v>1</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D55" s="15"/>
+      <c r="E55" s="12" t="s">
+        <v>47</v>
+      </c>
       <c r="F55" s="4"/>
-      <c r="G55" s="4"/>
-      <c r="H55" s="4"/>
+      <c r="G55" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="H55" s="12" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="56" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A56" s="15">
-        <v>401</v>
+        <v>307</v>
       </c>
       <c r="B56" s="15">
-        <v>1</v>
-      </c>
-      <c r="C56" s="6" t="s">
-        <v>19</v>
+        <v>2</v>
+      </c>
+      <c r="C56" s="12" t="s">
+        <v>110</v>
       </c>
       <c r="D56" s="15"/>
       <c r="E56" s="12" t="s">
-        <v>20</v>
+        <v>43</v>
       </c>
       <c r="F56" s="26" t="s">
-        <v>133</v>
-      </c>
-      <c r="G56" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="H56" s="26" t="s">
-        <v>133</v>
+        <v>109</v>
+      </c>
+      <c r="G56" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="H56" s="12" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="57" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A57" s="15">
-        <v>405</v>
+        <v>308</v>
       </c>
       <c r="B57" s="15">
-        <v>1</v>
-      </c>
-      <c r="C57" s="6" t="s">
-        <v>21</v>
+        <v>4</v>
+      </c>
+      <c r="C57" s="12" t="s">
+        <v>111</v>
       </c>
       <c r="D57" s="15"/>
       <c r="E57" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="F57" s="26" t="s">
+        <v>112</v>
+      </c>
+      <c r="G57" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="H57" s="12" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A58" s="14"/>
+      <c r="B58" s="14"/>
+      <c r="C58" s="7"/>
+      <c r="D58" s="20"/>
+      <c r="E58" s="7"/>
+      <c r="F58" s="4"/>
+      <c r="G58" s="4"/>
+      <c r="H58" s="4"/>
+    </row>
+    <row r="59" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A59" s="14"/>
+      <c r="B59" s="14"/>
+      <c r="C59" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D59" s="16"/>
+      <c r="E59" s="5"/>
+      <c r="F59" s="4"/>
+      <c r="G59" s="4"/>
+      <c r="H59" s="4"/>
+    </row>
+    <row r="60" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A60" s="15">
+        <v>401</v>
+      </c>
+      <c r="B60" s="15">
+        <v>1</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D60" s="15"/>
+      <c r="E60" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F60" s="26" t="s">
+        <v>139</v>
+      </c>
+      <c r="G60" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="H60" s="26" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A61" s="15">
+        <v>405</v>
+      </c>
+      <c r="B61" s="15">
+        <v>1</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D61" s="15"/>
+      <c r="E61" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="F57" s="26" t="s">
+      <c r="F61" s="26" t="s">
         <v>127</v>
       </c>
-      <c r="G57" s="12" t="s">
+      <c r="G61" s="12" t="s">
         <v>126</v>
       </c>
-      <c r="H57" s="4"/>
-    </row>
-    <row r="59" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="24" t="s">
+      <c r="H61" s="4"/>
+    </row>
+    <row r="63" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="24" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="60" spans="1:8" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="24"/>
-      <c r="B60" s="2">
-        <v>1</v>
-      </c>
-      <c r="C60" s="25" t="s">
+    <row r="64" spans="1:8" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="24"/>
+      <c r="B64" s="2">
+        <v>1</v>
+      </c>
+      <c r="C64" s="25" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="61" spans="1:8" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="24"/>
-      <c r="B61" s="2">
+    <row r="65" spans="1:3" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="24"/>
+      <c r="B65" s="2">
         <v>2</v>
       </c>
-      <c r="C61" s="25" t="s">
+      <c r="C65" s="25" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="62" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B62" s="2">
+    <row r="66" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B66" s="2">
         <v>3</v>
       </c>
-      <c r="C62" s="29" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="63" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B63" s="2">
+      <c r="C66" s="29" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B67" s="2">
         <v>4</v>
       </c>
-      <c r="C63" s="30" t="s">
+      <c r="C67" s="30" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="64" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B64" s="2">
+    <row r="68" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B68" s="2">
         <v>5</v>
       </c>
-      <c r="C64" s="30" t="s">
+      <c r="C68" s="30" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="65" spans="2:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B65" s="2">
+    <row r="69" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B69" s="2">
         <v>6</v>
       </c>
-      <c r="C65" s="30" t="s">
+      <c r="C69" s="30" t="s">
         <v>59</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B70" s="2">
+        <v>7</v>
+      </c>
+      <c r="C70" s="29" t="s">
+        <v>141</v>
       </c>
     </row>
   </sheetData>
@@ -2056,9 +2175,10 @@
     <hyperlink ref="F10" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="F9" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
     <hyperlink ref="F8" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="F18" r:id="rId4" xr:uid="{BF0182E4-427E-4CC9-9A79-B8FDFF700EB3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="72" fitToHeight="0" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId4"/>
+  <pageSetup scale="72" fitToHeight="0" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId5"/>
   <headerFooter>
     <oddFooter>Page &amp;P of &amp;N</oddFooter>
   </headerFooter>

</xml_diff>